<commit_message>
final fix scan route + dashboard
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -413,50 +413,94 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>uid</t>
+          <t>UID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>time</t>
+          <t>Time</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>Date</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>77146475</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Nikhil</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>10:36:25</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>91285723</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Abhishek</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>01:49:32</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>10:35:58</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1409145362</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Animesh</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>10:34:56</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>

</xml_diff>